<commit_message>
Added Connolly Tau calculation
The tortuosity analysis now measures both the Connolly and Lee-Richards tortuosity.
</commit_message>
<xml_diff>
--- a/tests/xyz/Example_Rectangular_Pore/Example_Output_Files/PSD_Plot.xlsx
+++ b/tests/xyz/Example_Rectangular_Pore/Example_Output_Files/PSD_Plot.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/42c400a6d2268350/Penn/GitHub/PARSE/tests/xyz/Example_Rectangular_Pore/Example_Output_Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="8_{7149973D-7FBA-47E4-9186-8284705DD2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E4C110C-6CE6-440C-A3A0-9EC2B15990EF}"/>
+  <xr:revisionPtr revIDLastSave="174" documentId="8_{7149973D-7FBA-47E4-9186-8284705DD2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C5C53C7-D145-4B00-A6A5-32F814E4ED91}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D12CB501-9D5F-4141-A117-3B2D7216ADD7}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D12CB501-9D5F-4141-A117-3B2D7216ADD7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>